<commit_message>
Round 2 dropdown: switch to team's agreed 17-category list
After discussing Round 1, the team settled on a slimmed-down 17-category
list (dropping Advertising, Network Security Monitoring, Operations,
Retail & Digital Commerce, Servers, Verticals, Web Tools & Plugins) for
what labelers can actually pick in Round 2. Added ROUND_CATEGORY_OVERRIDES
to make_labeling_workbook.py so a round's dropdown can diverge from its
sampled ProductSeries values, regenerated product_sample_round2.xlsx with
it, and documented scope (Round 2 labeling UI only -- sampling, answer
keys, and Round 1 are untouched) in the README.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/output/product_sample_round2.xlsx
+++ b/data/output/product_sample_round2.xlsx
@@ -2371,7 +2371,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid ProductSeries" error="Please choose a value from the dropdown list." type="list">
-      <formula1>='Category List'!$A$2:$A$25</formula1>
+      <formula1>='Category List'!$A$2:$A$18</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2384,7 +2384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2400,168 +2400,119 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Advertising</t>
+          <t>Collaborate Design &amp; Publish</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Collaborate Design &amp; Publish</t>
+          <t>Communications</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Communications</t>
+          <t>Customer Service</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Customer Service</t>
+          <t>Data Management Business Intelligence &amp; Analytics</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Data Management Business Intelligence &amp; Analytics</t>
+          <t>Enterprise Business Solution</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Enterprise Business Solution</t>
+          <t>Financial Management &amp; GRC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Financial Management &amp; GRC</t>
+          <t>Hardware</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Human Capital Management</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Human Capital Management</t>
+          <t>IT Development/Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IT Development/Infrastructure</t>
+          <t>IT Security Information</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IT Security Information</t>
+          <t>Marketing</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Network Security Monitoring</t>
+          <t>Sales</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Security Devices</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Service Management</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Retail &amp; Digital Commerce</t>
+          <t>Storage</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Security Devices</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Servers</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Service Management</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
           <t>Supply Chain Management</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Verticals</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Web Tools &amp; Plugins</t>
         </is>
       </c>
     </row>

</xml_diff>